<commit_message>
done, but it is really bad!
</commit_message>
<xml_diff>
--- a/code/crosswords/document/letter_distribution.xlsx
+++ b/code/crosswords/document/letter_distribution.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" state="visible" r:id="rId2"/>
@@ -13,6 +13,7 @@
     <sheet name="Planilha3" sheetId="3" state="visible" r:id="rId4"/>
     <sheet name="Planilha4" sheetId="4" state="visible" r:id="rId5"/>
     <sheet name="Planilha5" sheetId="5" state="visible" r:id="rId6"/>
+    <sheet name="Planilha6" sheetId="6" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1389" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1490" uniqueCount="73">
   <si>
     <t xml:space="preserve">interessante</t>
   </si>
@@ -237,6 +238,12 @@
   </si>
   <si>
     <t xml:space="preserve">interesse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">p</t>
   </si>
 </sst>
 </file>
@@ -28630,4 +28637,453 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Página &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:N14"/>
+  <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="1" style="0" width="3.23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="15" style="0" width="9.14"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="8"/>
+      <c r="B1" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="K1" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="N1" s="8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="H2" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="I2" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="L2" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="M2" s="8"/>
+      <c r="N2" s="8"/>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
+      <c r="L3" s="8"/>
+      <c r="M3" s="8"/>
+      <c r="N3" s="8"/>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="F4" s="8"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I4" s="8"/>
+      <c r="J4" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="L4" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="M4" s="8"/>
+      <c r="N4" s="8"/>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="I5" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="K5" s="8"/>
+      <c r="L5" s="8"/>
+      <c r="M5" s="8"/>
+      <c r="N5" s="8"/>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="I6" s="8"/>
+      <c r="J6" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="K6" s="8"/>
+      <c r="L6" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="M6" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="N6" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="I8" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="J8" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="K8" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="L8" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="L9" s="8"/>
+      <c r="M9" s="8"/>
+      <c r="N9" s="8" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
+      <c r="K10" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="L10" s="8"/>
+      <c r="M10" s="8"/>
+      <c r="N10" s="8" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="B11" s="8"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="I11" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="K11" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="L11" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="M11" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="N11" s="8" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="B12" s="8"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+      <c r="K12" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="L12" s="8"/>
+      <c r="M12" s="8"/>
+      <c r="N12" s="8" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="H13" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I13" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="J13" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="K13" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="L13" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="M13" s="8"/>
+      <c r="N13" s="8"/>
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="8"/>
+      <c r="K14" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="L14" s="8"/>
+      <c r="M14" s="8"/>
+      <c r="N14" s="8"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Página &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>